<commit_message>
feat(so): update template files
</commit_message>
<xml_diff>
--- a/document-merge-service/kt_so/templatefiles/vorpruefung-baugesuche.xlsx
+++ b/document-merge-service/kt_so/templatefiles/vorpruefung-baugesuche.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\BJSVW\Agi\eBau\Dokumentenvorlagen\eBau\Systemvorlagen\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\BJSVW\Agi\eBau\Dokumentenvorlagen\eBau\Systemvorlagen\Release15\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{040EA5C4-6230-43D2-A265-79E2EA7C330E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD83D6DE-AE25-4178-9EC3-E98C158FAE1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29280" yWindow="330" windowWidth="27015" windowHeight="15045" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-39765" yWindow="-1890" windowWidth="38700" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vorprüfung gross" sheetId="2" r:id="rId1"/>
@@ -1806,13 +1806,7 @@
     <t>Art. 49 Abs. 3</t>
   </si>
   <si>
-    <t>{{ BESCHREIBUNG_BAUVORHABEN }}</t>
-  </si>
-  <si>
     <t>{{ ADRESSE }}</t>
-  </si>
-  <si>
-    <t>Gesuchsteller/in</t>
   </si>
   <si>
     <t>Bauplatz (Adresse, Ort)</t>
@@ -1881,6 +1875,12 @@
       </rPr>
       <t>{{ HEUTE }}</t>
     </r>
+  </si>
+  <si>
+    <t>{{ KURZBESCHREIBUNG_BAUVORHABEN }}</t>
+  </si>
+  <si>
+    <t>Gesuchsteller/in (Bauherrschaft)</t>
   </si>
 </sst>
 </file>
@@ -2624,22 +2624,18 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2659,6 +2655,22 @@
     <xf numFmtId="16" fontId="1" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -2680,18 +2692,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -2974,38 +2974,38 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19783847-54E6-4BE1-8120-C3CEE97060F4}">
   <dimension ref="A1:L467"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="37.28515625" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" customWidth="1"/>
-    <col min="4" max="5" width="3.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.7109375" customWidth="1"/>
-    <col min="9" max="9" width="7.7109375" customWidth="1"/>
+    <col min="1" max="1" width="37.26953125" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" customWidth="1"/>
+    <col min="3" max="3" width="9.54296875" customWidth="1"/>
+    <col min="4" max="5" width="3.7265625" customWidth="1"/>
+    <col min="6" max="6" width="4.26953125" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7265625" customWidth="1"/>
+    <col min="9" max="9" width="7.7265625" customWidth="1"/>
     <col min="10" max="10" width="56" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="164" t="s">
-        <v>346</v>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" s="140" t="s">
+        <v>344</v>
       </c>
       <c r="I1" s="2"/>
       <c r="J1" s="3"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="165" t="s">
-        <v>347</v>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="141" t="s">
+        <v>345</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="5"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="I3" s="4"/>
       <c r="J3" s="5"/>
     </row>
-    <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
@@ -3019,7 +3019,7 @@
       <c r="I4" s="7"/>
       <c r="J4" s="7"/>
     </row>
-    <row r="5" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -3031,41 +3031,41 @@
       <c r="I5" s="9"/>
       <c r="J5" s="9"/>
     </row>
-    <row r="6" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
-        <v>344</v>
-      </c>
-      <c r="B6" s="166" t="s">
-        <v>348</v>
-      </c>
-      <c r="C6" s="167"/>
-      <c r="D6" s="167"/>
-      <c r="E6" s="167"/>
-      <c r="F6" s="167"/>
-      <c r="G6" s="167"/>
-      <c r="H6" s="167"/>
+        <v>352</v>
+      </c>
+      <c r="B6" s="142" t="s">
+        <v>346</v>
+      </c>
+      <c r="C6" s="143"/>
+      <c r="D6" s="143"/>
+      <c r="E6" s="143"/>
+      <c r="F6" s="143"/>
+      <c r="G6" s="143"/>
+      <c r="H6" s="143"/>
       <c r="I6" s="11"/>
       <c r="J6" s="11" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="168" t="s">
-        <v>342</v>
-      </c>
-      <c r="C7" s="169"/>
-      <c r="D7" s="169"/>
-      <c r="E7" s="169"/>
-      <c r="F7" s="169"/>
-      <c r="G7" s="169"/>
-      <c r="H7" s="169"/>
-      <c r="I7" s="169"/>
+      <c r="B7" s="144" t="s">
+        <v>351</v>
+      </c>
+      <c r="C7" s="145"/>
+      <c r="D7" s="145"/>
+      <c r="E7" s="145"/>
+      <c r="F7" s="145"/>
+      <c r="G7" s="145"/>
+      <c r="H7" s="145"/>
+      <c r="I7" s="145"/>
       <c r="J7" s="13"/>
     </row>
-    <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="12" t="s">
         <v>1</v>
       </c>
@@ -3081,25 +3081,25 @@
       <c r="I8" s="14"/>
       <c r="J8" s="13"/>
     </row>
-    <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="12" t="s">
-        <v>345</v>
-      </c>
-      <c r="B9" s="168" t="s">
         <v>343</v>
       </c>
-      <c r="C9" s="169"/>
-      <c r="D9" s="169"/>
-      <c r="E9" s="169"/>
-      <c r="F9" s="169"/>
-      <c r="G9" s="169"/>
-      <c r="H9" s="169"/>
-      <c r="I9" s="169"/>
+      <c r="B9" s="144" t="s">
+        <v>342</v>
+      </c>
+      <c r="C9" s="145"/>
+      <c r="D9" s="145"/>
+      <c r="E9" s="145"/>
+      <c r="F9" s="145"/>
+      <c r="G9" s="145"/>
+      <c r="H9" s="145"/>
+      <c r="I9" s="145"/>
       <c r="J9" s="13"/>
     </row>
-    <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="12" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B10" s="16" t="s">
         <v>4</v>
@@ -3114,12 +3114,12 @@
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
       <c r="J10" s="139" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="12" t="s">
         <v>350</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
-        <v>352</v>
       </c>
       <c r="B11" s="14" t="s">
         <v>6</v>
@@ -3133,7 +3133,7 @@
       <c r="I11" s="14"/>
       <c r="J11" s="13"/>
     </row>
-    <row r="12" spans="1:12" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="5.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -3145,34 +3145,34 @@
       <c r="I12" s="9"/>
       <c r="J12" s="9"/>
     </row>
-    <row r="13" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="148" t="s">
+    <row r="13" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="146" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="150" t="s">
+      <c r="B13" s="148" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="152" t="s">
+      <c r="C13" s="150" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="153" t="s">
+      <c r="D13" s="151" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="154"/>
-      <c r="F13" s="155"/>
-      <c r="G13" s="156"/>
-      <c r="H13" s="154"/>
+      <c r="E13" s="152"/>
+      <c r="F13" s="153"/>
+      <c r="G13" s="154"/>
+      <c r="H13" s="152"/>
       <c r="I13" s="18"/>
-      <c r="J13" s="140" t="s">
+      <c r="J13" s="155" t="s">
         <v>11</v>
       </c>
-      <c r="K13" s="142"/>
-      <c r="L13" s="142"/>
-    </row>
-    <row r="14" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="149"/>
-      <c r="B14" s="151"/>
-      <c r="C14" s="149"/>
+      <c r="K13" s="157"/>
+      <c r="L13" s="157"/>
+    </row>
+    <row r="14" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="147"/>
+      <c r="B14" s="149"/>
+      <c r="C14" s="147"/>
       <c r="D14" s="19" t="s">
         <v>12</v>
       </c>
@@ -3191,25 +3191,25 @@
       <c r="I14" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="J14" s="141"/>
-      <c r="K14" s="143"/>
-      <c r="L14" s="143"/>
-    </row>
-    <row r="15" spans="1:12" s="9" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="144" t="s">
+      <c r="J14" s="156"/>
+      <c r="K14" s="158"/>
+      <c r="L14" s="158"/>
+    </row>
+    <row r="15" spans="1:12" s="9" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="159" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="145"/>
-      <c r="C15" s="145"/>
-      <c r="D15" s="145"/>
-      <c r="E15" s="145"/>
-      <c r="F15" s="145"/>
-      <c r="G15" s="145"/>
-      <c r="H15" s="145"/>
-      <c r="I15" s="145"/>
-      <c r="J15" s="145"/>
-    </row>
-    <row r="16" spans="1:12" s="25" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="160"/>
+      <c r="C15" s="160"/>
+      <c r="D15" s="160"/>
+      <c r="E15" s="160"/>
+      <c r="F15" s="160"/>
+      <c r="G15" s="160"/>
+      <c r="H15" s="160"/>
+      <c r="I15" s="160"/>
+      <c r="J15" s="160"/>
+    </row>
+    <row r="16" spans="1:12" s="25" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="21" t="s">
         <v>19</v>
       </c>
@@ -3223,7 +3223,7 @@
       <c r="I16" s="23"/>
       <c r="J16" s="23"/>
     </row>
-    <row r="17" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="26" t="s">
         <v>20</v>
       </c>
@@ -3245,7 +3245,7 @@
       <c r="I17" s="31"/>
       <c r="J17" s="32"/>
     </row>
-    <row r="18" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="26" t="s">
         <v>23</v>
       </c>
@@ -3267,7 +3267,7 @@
       <c r="I18" s="31"/>
       <c r="J18" s="32"/>
     </row>
-    <row r="19" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="34" t="s">
         <v>24</v>
       </c>
@@ -3289,7 +3289,7 @@
       <c r="I19" s="31"/>
       <c r="J19" s="32"/>
     </row>
-    <row r="20" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="34" t="s">
         <v>26</v>
       </c>
@@ -3311,7 +3311,7 @@
       <c r="I20" s="31"/>
       <c r="J20" s="32"/>
     </row>
-    <row r="21" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="34" t="s">
         <v>27</v>
       </c>
@@ -3333,7 +3333,7 @@
       <c r="I21" s="31"/>
       <c r="J21" s="32"/>
     </row>
-    <row r="22" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="26" t="s">
         <v>28</v>
       </c>
@@ -3355,7 +3355,7 @@
       <c r="I22" s="31"/>
       <c r="J22" s="32"/>
     </row>
-    <row r="23" spans="1:10" s="35" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" s="35" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="34" t="s">
         <v>30</v>
       </c>
@@ -3377,7 +3377,7 @@
       <c r="I23" s="31"/>
       <c r="J23" s="32"/>
     </row>
-    <row r="24" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="26" t="s">
         <v>32</v>
       </c>
@@ -3399,7 +3399,7 @@
       <c r="I24" s="39"/>
       <c r="J24" s="32"/>
     </row>
-    <row r="25" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="26" t="s">
         <v>34</v>
       </c>
@@ -3421,7 +3421,7 @@
       <c r="I25" s="31"/>
       <c r="J25" s="32"/>
     </row>
-    <row r="26" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="26" t="s">
         <v>35</v>
       </c>
@@ -3443,7 +3443,7 @@
       <c r="I26" s="31"/>
       <c r="J26" s="32"/>
     </row>
-    <row r="27" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="26" t="s">
         <v>37</v>
       </c>
@@ -3465,7 +3465,7 @@
       <c r="I27" s="31"/>
       <c r="J27" s="32"/>
     </row>
-    <row r="28" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="26" t="s">
         <v>38</v>
       </c>
@@ -3487,7 +3487,7 @@
       <c r="I28" s="31"/>
       <c r="J28" s="32"/>
     </row>
-    <row r="29" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="40" t="s">
         <v>40</v>
       </c>
@@ -3511,7 +3511,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="26" t="s">
         <v>43</v>
       </c>
@@ -3533,7 +3533,7 @@
       <c r="I30" s="31"/>
       <c r="J30" s="32"/>
     </row>
-    <row r="31" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="26" t="s">
         <v>45</v>
       </c>
@@ -3553,7 +3553,7 @@
       <c r="I31" s="31"/>
       <c r="J31" s="32"/>
     </row>
-    <row r="32" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="41" t="s">
         <v>48</v>
       </c>
@@ -3569,7 +3569,7 @@
       <c r="I32" s="31"/>
       <c r="J32" s="32"/>
     </row>
-    <row r="33" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="41" t="s">
         <v>50</v>
       </c>
@@ -3583,7 +3583,7 @@
       <c r="I33" s="31"/>
       <c r="J33" s="32"/>
     </row>
-    <row r="34" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="41" t="s">
         <v>51</v>
       </c>
@@ -3597,7 +3597,7 @@
       <c r="I34" s="31"/>
       <c r="J34" s="32"/>
     </row>
-    <row r="35" spans="1:10" s="25" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" s="25" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="21" t="s">
         <v>52</v>
       </c>
@@ -3611,7 +3611,7 @@
       <c r="I35" s="23"/>
       <c r="J35" s="23"/>
     </row>
-    <row r="36" spans="1:10" s="47" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" s="47" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="43" t="s">
         <v>53</v>
       </c>
@@ -3625,7 +3625,7 @@
       <c r="I36" s="46"/>
       <c r="J36" s="45"/>
     </row>
-    <row r="37" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="26" t="s">
         <v>54</v>
       </c>
@@ -3645,7 +3645,7 @@
       <c r="I37" s="31"/>
       <c r="J37" s="32"/>
     </row>
-    <row r="38" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="26" t="s">
         <v>56</v>
       </c>
@@ -3665,7 +3665,7 @@
       <c r="I38" s="31"/>
       <c r="J38" s="32"/>
     </row>
-    <row r="39" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="26" t="s">
         <v>58</v>
       </c>
@@ -3687,7 +3687,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="26" t="s">
         <v>60</v>
       </c>
@@ -3709,7 +3709,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="26" t="s">
         <v>61</v>
       </c>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="J41" s="32"/>
     </row>
-    <row r="42" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="41" t="s">
         <v>63</v>
       </c>
@@ -3751,7 +3751,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="43" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="26" t="s">
         <v>67</v>
       </c>
@@ -3771,7 +3771,7 @@
       <c r="I43" s="31"/>
       <c r="J43" s="32"/>
     </row>
-    <row r="44" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="26" t="s">
         <v>69</v>
       </c>
@@ -3791,7 +3791,7 @@
       <c r="I44" s="31"/>
       <c r="J44" s="32"/>
     </row>
-    <row r="45" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="26" t="s">
         <v>71</v>
       </c>
@@ -3811,7 +3811,7 @@
       <c r="I45" s="31"/>
       <c r="J45" s="32"/>
     </row>
-    <row r="46" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="26" t="s">
         <v>72</v>
       </c>
@@ -3831,7 +3831,7 @@
       <c r="I46" s="31"/>
       <c r="J46" s="32"/>
     </row>
-    <row r="47" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="26" t="s">
         <v>74</v>
       </c>
@@ -3851,7 +3851,7 @@
       <c r="I47" s="31"/>
       <c r="J47" s="32"/>
     </row>
-    <row r="48" spans="1:10" s="47" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" s="47" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="43" t="s">
         <v>76</v>
       </c>
@@ -3865,7 +3865,7 @@
       <c r="I48" s="46"/>
       <c r="J48" s="45"/>
     </row>
-    <row r="49" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="26" t="s">
         <v>77</v>
       </c>
@@ -3885,7 +3885,7 @@
       <c r="I49" s="31"/>
       <c r="J49" s="32"/>
     </row>
-    <row r="50" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="50" t="s">
         <v>79</v>
       </c>
@@ -3905,7 +3905,7 @@
       </c>
       <c r="J50" s="32"/>
     </row>
-    <row r="51" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="51" t="s">
         <v>82</v>
       </c>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="J51" s="56"/>
     </row>
-    <row r="52" spans="1:10" s="35" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" s="35" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="34" t="s">
         <v>84</v>
       </c>
@@ -3947,7 +3947,7 @@
       </c>
       <c r="J52" s="32"/>
     </row>
-    <row r="53" spans="1:10" s="35" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" s="35" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="34" t="s">
         <v>86</v>
       </c>
@@ -3967,7 +3967,7 @@
       <c r="I53" s="31"/>
       <c r="J53" s="32"/>
     </row>
-    <row r="54" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="40" t="s">
         <v>88</v>
       </c>
@@ -3983,7 +3983,7 @@
       <c r="I54" s="55"/>
       <c r="J54" s="56"/>
     </row>
-    <row r="55" spans="1:10" s="35" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" s="35" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="51" t="s">
         <v>89</v>
       </c>
@@ -4003,7 +4003,7 @@
       <c r="I55" s="39"/>
       <c r="J55" s="60"/>
     </row>
-    <row r="56" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="61" t="s">
         <v>90</v>
       </c>
@@ -4023,7 +4023,7 @@
       <c r="I56" s="31"/>
       <c r="J56" s="32"/>
     </row>
-    <row r="57" spans="1:10" s="47" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" s="47" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="43" t="s">
         <v>91</v>
       </c>
@@ -4037,7 +4037,7 @@
       <c r="I57" s="46"/>
       <c r="J57" s="45"/>
     </row>
-    <row r="58" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="26" t="s">
         <v>92</v>
       </c>
@@ -4059,7 +4059,7 @@
       </c>
       <c r="J58" s="32"/>
     </row>
-    <row r="59" spans="1:10" s="35" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" s="35" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="62" t="s">
         <v>94</v>
       </c>
@@ -4081,7 +4081,7 @@
       </c>
       <c r="J59" s="32"/>
     </row>
-    <row r="60" spans="1:10" s="35" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" s="35" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="61" t="s">
         <v>96</v>
       </c>
@@ -4101,21 +4101,21 @@
       <c r="I60" s="31"/>
       <c r="J60" s="32"/>
     </row>
-    <row r="61" spans="1:10" s="25" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="146" t="s">
+    <row r="61" spans="1:10" s="25" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="161" t="s">
         <v>98</v>
       </c>
-      <c r="B61" s="147"/>
-      <c r="C61" s="147"/>
-      <c r="D61" s="147"/>
-      <c r="E61" s="147"/>
-      <c r="F61" s="147"/>
-      <c r="G61" s="147"/>
-      <c r="H61" s="147"/>
-      <c r="I61" s="147"/>
-      <c r="J61" s="147"/>
-    </row>
-    <row r="62" spans="1:10" s="25" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B61" s="162"/>
+      <c r="C61" s="162"/>
+      <c r="D61" s="162"/>
+      <c r="E61" s="162"/>
+      <c r="F61" s="162"/>
+      <c r="G61" s="162"/>
+      <c r="H61" s="162"/>
+      <c r="I61" s="162"/>
+      <c r="J61" s="162"/>
+    </row>
+    <row r="62" spans="1:10" s="25" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="21" t="s">
         <v>99</v>
       </c>
@@ -4129,7 +4129,7 @@
       <c r="I62" s="23"/>
       <c r="J62" s="23"/>
     </row>
-    <row r="63" spans="1:10" s="33" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" s="33" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="62" t="s">
         <v>100</v>
       </c>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="J63" s="32"/>
     </row>
-    <row r="64" spans="1:10" s="33" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" s="33" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="62" t="s">
         <v>103</v>
       </c>
@@ -4171,7 +4171,7 @@
       <c r="I64" s="55"/>
       <c r="J64" s="32"/>
     </row>
-    <row r="65" spans="1:10" s="33" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" s="33" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="62" t="s">
         <v>106</v>
       </c>
@@ -4193,7 +4193,7 @@
       </c>
       <c r="J65" s="32"/>
     </row>
-    <row r="66" spans="1:10" s="33" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" s="33" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="62" t="s">
         <v>108</v>
       </c>
@@ -4213,7 +4213,7 @@
       <c r="I66" s="55"/>
       <c r="J66" s="32"/>
     </row>
-    <row r="67" spans="1:10" s="33" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" s="33" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="62" t="s">
         <v>110</v>
       </c>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="J67" s="32"/>
     </row>
-    <row r="68" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="62" t="s">
         <v>112</v>
       </c>
@@ -4255,7 +4255,7 @@
       <c r="I68" s="55"/>
       <c r="J68" s="32"/>
     </row>
-    <row r="69" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="62" t="s">
         <v>114</v>
       </c>
@@ -4275,7 +4275,7 @@
       <c r="I69" s="55"/>
       <c r="J69" s="32"/>
     </row>
-    <row r="70" spans="1:10" s="33" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" s="33" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="62" t="s">
         <v>115</v>
       </c>
@@ -4295,7 +4295,7 @@
       <c r="I70" s="55"/>
       <c r="J70" s="32"/>
     </row>
-    <row r="71" spans="1:10" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="62" t="s">
         <v>116</v>
       </c>
@@ -4317,7 +4317,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="72" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="62" t="s">
         <v>119</v>
       </c>
@@ -4337,7 +4337,7 @@
       <c r="I72" s="55"/>
       <c r="J72" s="32"/>
     </row>
-    <row r="73" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="40" t="s">
         <v>121</v>
       </c>
@@ -4357,7 +4357,7 @@
       <c r="I73" s="55"/>
       <c r="J73" s="32"/>
     </row>
-    <row r="74" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" s="33" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="40" t="s">
         <v>122</v>
       </c>
@@ -4371,7 +4371,7 @@
       <c r="I74" s="55"/>
       <c r="J74" s="32"/>
     </row>
-    <row r="75" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="26" t="s">
         <v>123</v>
       </c>
@@ -4391,7 +4391,7 @@
       <c r="I75" s="31"/>
       <c r="J75" s="32"/>
     </row>
-    <row r="76" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="26" t="s">
         <v>124</v>
       </c>
@@ -4411,7 +4411,7 @@
       <c r="I76" s="31"/>
       <c r="J76" s="32"/>
     </row>
-    <row r="77" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="26" t="s">
         <v>125</v>
       </c>
@@ -4435,7 +4435,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="78" spans="1:10" s="35" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" s="35" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="34" t="s">
         <v>128</v>
       </c>
@@ -4459,7 +4459,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="79" spans="1:10" s="35" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" s="35" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="34" t="s">
         <v>131</v>
       </c>
@@ -4479,7 +4479,7 @@
       <c r="I79" s="31"/>
       <c r="J79" s="32"/>
     </row>
-    <row r="80" spans="1:10" s="35" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" s="35" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="26" t="s">
         <v>132</v>
       </c>
@@ -4499,7 +4499,7 @@
       <c r="I80" s="31"/>
       <c r="J80" s="32"/>
     </row>
-    <row r="81" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="26" t="s">
         <v>134</v>
       </c>
@@ -4519,7 +4519,7 @@
       <c r="I81" s="31"/>
       <c r="J81" s="32"/>
     </row>
-    <row r="82" spans="1:10" s="70" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" s="70" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="34" t="s">
         <v>135</v>
       </c>
@@ -4541,7 +4541,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="83" spans="1:10" s="70" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" s="70" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="34" t="s">
         <v>139</v>
       </c>
@@ -4563,7 +4563,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="84" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="34" t="s">
         <v>142</v>
       </c>
@@ -4583,7 +4583,7 @@
       <c r="I84" s="31"/>
       <c r="J84" s="32"/>
     </row>
-    <row r="85" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="26" t="s">
         <v>144</v>
       </c>
@@ -4605,7 +4605,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="86" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="26" t="s">
         <v>147</v>
       </c>
@@ -4623,7 +4623,7 @@
       <c r="I86" s="31"/>
       <c r="J86" s="71"/>
     </row>
-    <row r="87" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="41" t="s">
         <v>148</v>
       </c>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="J87" s="32"/>
     </row>
-    <row r="88" spans="1:10" s="75" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" s="75" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="21" t="s">
         <v>149</v>
       </c>
@@ -4653,7 +4653,7 @@
       <c r="I88" s="74"/>
       <c r="J88" s="21"/>
     </row>
-    <row r="89" spans="1:10" s="47" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" s="47" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="43" t="s">
         <v>150</v>
       </c>
@@ -4667,7 +4667,7 @@
       <c r="I89" s="46"/>
       <c r="J89" s="45"/>
     </row>
-    <row r="90" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="40" t="s">
         <v>151</v>
       </c>
@@ -4681,7 +4681,7 @@
       <c r="I90" s="55"/>
       <c r="J90" s="56"/>
     </row>
-    <row r="91" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="61" t="s">
         <v>152</v>
       </c>
@@ -4699,7 +4699,7 @@
       <c r="I91" s="39"/>
       <c r="J91" s="60"/>
     </row>
-    <row r="92" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="26" t="s">
         <v>153</v>
       </c>
@@ -4717,7 +4717,7 @@
       <c r="I92" s="39"/>
       <c r="J92" s="32"/>
     </row>
-    <row r="93" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="26" t="s">
         <v>154</v>
       </c>
@@ -4735,7 +4735,7 @@
       <c r="I93" s="39"/>
       <c r="J93" s="32"/>
     </row>
-    <row r="94" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="61" t="s">
         <v>155</v>
       </c>
@@ -4753,7 +4753,7 @@
       <c r="I94" s="39"/>
       <c r="J94" s="32"/>
     </row>
-    <row r="95" spans="1:10" s="35" customFormat="1" ht="36.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" s="35" customFormat="1" ht="37" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="62" t="s">
         <v>156</v>
       </c>
@@ -4775,7 +4775,7 @@
       <c r="I95" s="79"/>
       <c r="J95" s="56"/>
     </row>
-    <row r="96" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="40" t="s">
         <v>158</v>
       </c>
@@ -4789,7 +4789,7 @@
       <c r="I96" s="55"/>
       <c r="J96" s="56"/>
     </row>
-    <row r="97" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="61" t="s">
         <v>152</v>
       </c>
@@ -4807,7 +4807,7 @@
       <c r="I97" s="39"/>
       <c r="J97" s="60"/>
     </row>
-    <row r="98" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="26" t="s">
         <v>153</v>
       </c>
@@ -4825,7 +4825,7 @@
       <c r="I98" s="39"/>
       <c r="J98" s="32"/>
     </row>
-    <row r="99" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="26" t="s">
         <v>154</v>
       </c>
@@ -4843,7 +4843,7 @@
       <c r="I99" s="39"/>
       <c r="J99" s="32"/>
     </row>
-    <row r="100" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="61" t="s">
         <v>155</v>
       </c>
@@ -4861,7 +4861,7 @@
       <c r="I100" s="39"/>
       <c r="J100" s="32"/>
     </row>
-    <row r="101" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="62" t="s">
         <v>159</v>
       </c>
@@ -4881,7 +4881,7 @@
       <c r="I101" s="79"/>
       <c r="J101" s="56"/>
     </row>
-    <row r="102" spans="1:10" s="35" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" s="35" customFormat="1" ht="27.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="62" t="s">
         <v>161</v>
       </c>
@@ -4901,7 +4901,7 @@
       <c r="I102" s="79"/>
       <c r="J102" s="56"/>
     </row>
-    <row r="103" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="62" t="s">
         <v>163</v>
       </c>
@@ -4915,7 +4915,7 @@
       <c r="I103" s="79"/>
       <c r="J103" s="56"/>
     </row>
-    <row r="104" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="50" t="s">
         <v>164</v>
       </c>
@@ -4935,7 +4935,7 @@
       <c r="I104" s="39"/>
       <c r="J104" s="60"/>
     </row>
-    <row r="105" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="62" t="s">
         <v>166</v>
       </c>
@@ -4955,7 +4955,7 @@
       <c r="I105" s="79"/>
       <c r="J105" s="56"/>
     </row>
-    <row r="106" spans="1:10" s="35" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" s="35" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="83" t="s">
         <v>168</v>
       </c>
@@ -4979,7 +4979,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="107" spans="1:10" s="35" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" s="35" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" s="34" t="s">
         <v>171</v>
       </c>
@@ -5003,7 +5003,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="108" spans="1:10" s="35" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" s="35" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" s="84" t="s">
         <v>174</v>
       </c>
@@ -5027,7 +5027,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="109" spans="1:10" s="35" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" s="35" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="34" t="s">
         <v>176</v>
       </c>
@@ -5045,7 +5045,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="110" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="84"/>
       <c r="B110" s="36"/>
       <c r="C110" s="72"/>
@@ -5057,7 +5057,7 @@
       <c r="I110" s="31"/>
       <c r="J110" s="32"/>
     </row>
-    <row r="111" spans="1:10" s="47" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" s="47" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111" s="43" t="s">
         <v>178</v>
       </c>
@@ -5187,7 +5187,7 @@
       <c r="I117" s="39"/>
       <c r="J117" s="32"/>
     </row>
-    <row r="118" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118" s="26" t="s">
         <v>191</v>
       </c>
@@ -5207,7 +5207,7 @@
       <c r="I118" s="31"/>
       <c r="J118" s="32"/>
     </row>
-    <row r="119" spans="1:10" s="35" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10" s="35" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" s="34" t="s">
         <v>193</v>
       </c>
@@ -5227,7 +5227,7 @@
       <c r="I119" s="39"/>
       <c r="J119" s="32"/>
     </row>
-    <row r="120" spans="1:10" s="33" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10" s="33" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120" s="26" t="s">
         <v>195</v>
       </c>
@@ -5249,7 +5249,7 @@
       <c r="I120" s="31"/>
       <c r="J120" s="32"/>
     </row>
-    <row r="121" spans="1:10" s="47" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:10" s="47" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121" s="43" t="s">
         <v>197</v>
       </c>
@@ -5263,7 +5263,7 @@
       <c r="I121" s="46"/>
       <c r="J121" s="45"/>
     </row>
-    <row r="122" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" s="26" t="s">
         <v>198</v>
       </c>
@@ -5283,7 +5283,7 @@
       <c r="I122" s="31"/>
       <c r="J122" s="32"/>
     </row>
-    <row r="123" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="34" t="s">
         <v>200</v>
       </c>
@@ -5303,7 +5303,7 @@
       <c r="I123" s="39"/>
       <c r="J123" s="32"/>
     </row>
-    <row r="124" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" s="62" t="s">
         <v>202</v>
       </c>
@@ -5323,7 +5323,7 @@
       <c r="I124" s="39"/>
       <c r="J124" s="32"/>
     </row>
-    <row r="125" spans="1:10" s="35" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:10" s="35" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A125" s="62" t="s">
         <v>204</v>
       </c>
@@ -5337,7 +5337,7 @@
       <c r="I125" s="79"/>
       <c r="J125" s="56"/>
     </row>
-    <row r="126" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A126" s="50" t="s">
         <v>205</v>
       </c>
@@ -5355,7 +5355,7 @@
       <c r="I126" s="39"/>
       <c r="J126" s="60"/>
     </row>
-    <row r="127" spans="1:10" s="35" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:10" s="35" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A127" s="62" t="s">
         <v>206</v>
       </c>
@@ -5373,7 +5373,7 @@
       <c r="I127" s="39"/>
       <c r="J127" s="32"/>
     </row>
-    <row r="128" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A128" s="62" t="s">
         <v>207</v>
       </c>
@@ -5391,7 +5391,7 @@
       <c r="I128" s="39"/>
       <c r="J128" s="32"/>
     </row>
-    <row r="129" spans="1:10" s="35" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:10" s="35" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="62" t="s">
         <v>208</v>
       </c>
@@ -5407,7 +5407,7 @@
       <c r="I129" s="39"/>
       <c r="J129" s="32"/>
     </row>
-    <row r="130" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A130" s="34" t="s">
         <v>210</v>
       </c>
@@ -5427,7 +5427,7 @@
       <c r="I130" s="31"/>
       <c r="J130" s="32"/>
     </row>
-    <row r="131" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131" s="34"/>
       <c r="B131" s="27"/>
       <c r="C131" s="29"/>
@@ -5439,7 +5439,7 @@
       <c r="I131" s="31"/>
       <c r="J131" s="32"/>
     </row>
-    <row r="132" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A132" s="34"/>
       <c r="B132" s="27"/>
       <c r="C132" s="29"/>
@@ -5451,7 +5451,7 @@
       <c r="I132" s="31"/>
       <c r="J132" s="32"/>
     </row>
-    <row r="133" spans="1:10" s="47" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" s="47" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A133" s="43" t="s">
         <v>212</v>
       </c>
@@ -5465,7 +5465,7 @@
       <c r="I133" s="46"/>
       <c r="J133" s="45"/>
     </row>
-    <row r="134" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A134" s="26" t="s">
         <v>213</v>
       </c>
@@ -5505,7 +5505,7 @@
       <c r="I135" s="39"/>
       <c r="J135" s="60"/>
     </row>
-    <row r="136" spans="1:10" s="35" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:10" s="35" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="50" t="s">
         <v>216</v>
       </c>
@@ -5527,7 +5527,7 @@
       <c r="I136" s="39"/>
       <c r="J136" s="60"/>
     </row>
-    <row r="137" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A137" s="50" t="s">
         <v>218</v>
       </c>
@@ -5555,7 +5555,7 @@
       <c r="I137" s="39"/>
       <c r="J137" s="60"/>
     </row>
-    <row r="138" spans="1:10" s="35" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:10" s="35" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A138" s="34" t="s">
         <v>220</v>
       </c>
@@ -5573,7 +5573,7 @@
       <c r="I138" s="31"/>
       <c r="J138" s="32"/>
     </row>
-    <row r="139" spans="1:10" s="35" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:10" s="35" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A139" s="34" t="s">
         <v>221</v>
       </c>
@@ -5591,7 +5591,7 @@
       <c r="I139" s="39"/>
       <c r="J139" s="32"/>
     </row>
-    <row r="140" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A140" s="26" t="s">
         <v>222</v>
       </c>
@@ -5609,7 +5609,7 @@
       <c r="I140" s="39"/>
       <c r="J140" s="32"/>
     </row>
-    <row r="141" spans="1:10" s="35" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:10" s="35" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A141" s="34" t="s">
         <v>223</v>
       </c>
@@ -5627,7 +5627,7 @@
       <c r="I141" s="31"/>
       <c r="J141" s="32"/>
     </row>
-    <row r="142" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A142" s="26" t="s">
         <v>224</v>
       </c>
@@ -5649,7 +5649,7 @@
       <c r="I142" s="31"/>
       <c r="J142" s="32"/>
     </row>
-    <row r="143" spans="1:10" s="47" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:10" s="47" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A143" s="43" t="s">
         <v>225</v>
       </c>
@@ -5663,7 +5663,7 @@
       <c r="I143" s="46"/>
       <c r="J143" s="45"/>
     </row>
-    <row r="144" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A144" s="61" t="s">
         <v>226</v>
       </c>
@@ -5685,7 +5685,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="145" spans="1:10" s="35" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:10" s="35" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="34" t="s">
         <v>229</v>
       </c>
@@ -5705,7 +5705,7 @@
       <c r="I145" s="39"/>
       <c r="J145" s="32"/>
     </row>
-    <row r="146" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A146" s="40" t="s">
         <v>231</v>
       </c>
@@ -5729,7 +5729,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="147" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A147" s="26" t="s">
         <v>234</v>
       </c>
@@ -5749,7 +5749,7 @@
       <c r="I147" s="39"/>
       <c r="J147" s="32"/>
     </row>
-    <row r="148" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A148" s="61" t="s">
         <v>236</v>
       </c>
@@ -5771,7 +5771,7 @@
       <c r="I148" s="39"/>
       <c r="J148" s="60"/>
     </row>
-    <row r="149" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A149" s="40" t="s">
         <v>238</v>
       </c>
@@ -5793,7 +5793,7 @@
       <c r="I149" s="39"/>
       <c r="J149" s="32"/>
     </row>
-    <row r="150" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A150" s="40" t="s">
         <v>240</v>
       </c>
@@ -5813,7 +5813,7 @@
       <c r="I150" s="39"/>
       <c r="J150" s="32"/>
     </row>
-    <row r="151" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A151" s="40" t="s">
         <v>242</v>
       </c>
@@ -5835,7 +5835,7 @@
       <c r="I151" s="39"/>
       <c r="J151" s="32"/>
     </row>
-    <row r="152" spans="1:10" s="35" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:10" s="35" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A152" s="34" t="s">
         <v>243</v>
       </c>
@@ -5855,7 +5855,7 @@
       <c r="I152" s="31"/>
       <c r="J152" s="32"/>
     </row>
-    <row r="153" spans="1:10" s="47" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:10" s="47" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A153" s="43" t="s">
         <v>245</v>
       </c>
@@ -5869,7 +5869,7 @@
       <c r="I153" s="46"/>
       <c r="J153" s="45"/>
     </row>
-    <row r="154" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A154" s="26" t="s">
         <v>246</v>
       </c>
@@ -5889,7 +5889,7 @@
       <c r="I154" s="31"/>
       <c r="J154" s="32"/>
     </row>
-    <row r="155" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A155" s="26" t="s">
         <v>248</v>
       </c>
@@ -5909,7 +5909,7 @@
       <c r="I155" s="39"/>
       <c r="J155" s="32"/>
     </row>
-    <row r="156" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A156" s="26" t="s">
         <v>250</v>
       </c>
@@ -5985,7 +5985,7 @@
       <c r="I159" s="39"/>
       <c r="J159" s="32"/>
     </row>
-    <row r="160" spans="1:10" s="47" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:10" s="47" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A160" s="43" t="s">
         <v>258</v>
       </c>
@@ -5999,7 +5999,7 @@
       <c r="I160" s="46"/>
       <c r="J160" s="45"/>
     </row>
-    <row r="161" spans="1:10" s="35" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:10" s="35" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A161" s="34" t="s">
         <v>259</v>
       </c>
@@ -6019,7 +6019,7 @@
       <c r="I161" s="31"/>
       <c r="J161" s="32"/>
     </row>
-    <row r="162" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A162" s="26" t="s">
         <v>261</v>
       </c>
@@ -6041,7 +6041,7 @@
       <c r="I162" s="39"/>
       <c r="J162" s="32"/>
     </row>
-    <row r="163" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A163" s="40" t="s">
         <v>264</v>
       </c>
@@ -6055,7 +6055,7 @@
       <c r="I163" s="79"/>
       <c r="J163" s="56"/>
     </row>
-    <row r="164" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A164" s="61" t="s">
         <v>265</v>
       </c>
@@ -6075,7 +6075,7 @@
       <c r="I164" s="39"/>
       <c r="J164" s="60"/>
     </row>
-    <row r="165" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A165" s="26" t="s">
         <v>266</v>
       </c>
@@ -6133,7 +6133,7 @@
       <c r="I167" s="31"/>
       <c r="J167" s="32"/>
     </row>
-    <row r="168" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A168" s="26" t="s">
         <v>272</v>
       </c>
@@ -6155,7 +6155,7 @@
       <c r="I168" s="31"/>
       <c r="J168" s="32"/>
     </row>
-    <row r="169" spans="1:10" s="35" customFormat="1" ht="36.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:10" s="35" customFormat="1" ht="37" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A169" s="34" t="s">
         <v>273</v>
       </c>
@@ -6175,7 +6175,7 @@
       <c r="I169" s="31"/>
       <c r="J169" s="32"/>
     </row>
-    <row r="170" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A170" s="40" t="s">
         <v>275</v>
       </c>
@@ -6197,7 +6197,7 @@
       <c r="I170" s="39"/>
       <c r="J170" s="32"/>
     </row>
-    <row r="171" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A171" s="26" t="s">
         <v>277</v>
       </c>
@@ -6217,7 +6217,7 @@
       <c r="I171" s="31"/>
       <c r="J171" s="32"/>
     </row>
-    <row r="172" spans="1:10" s="47" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:10" s="47" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A172" s="43" t="s">
         <v>278</v>
       </c>
@@ -6231,7 +6231,7 @@
       <c r="I172" s="46"/>
       <c r="J172" s="45"/>
     </row>
-    <row r="173" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A173" s="26" t="s">
         <v>279</v>
       </c>
@@ -6251,7 +6251,7 @@
       <c r="I173" s="39"/>
       <c r="J173" s="32"/>
     </row>
-    <row r="174" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A174" s="40" t="s">
         <v>281</v>
       </c>
@@ -6271,7 +6271,7 @@
       <c r="I174" s="39"/>
       <c r="J174" s="32"/>
     </row>
-    <row r="175" spans="1:10" s="35" customFormat="1" ht="36.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:10" s="35" customFormat="1" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="62" t="s">
         <v>283</v>
       </c>
@@ -6291,7 +6291,7 @@
       <c r="I175" s="39"/>
       <c r="J175" s="32"/>
     </row>
-    <row r="176" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A176" s="40" t="s">
         <v>285</v>
       </c>
@@ -6311,7 +6311,7 @@
       <c r="I176" s="39"/>
       <c r="J176" s="32"/>
     </row>
-    <row r="177" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A177" s="40" t="s">
         <v>287</v>
       </c>
@@ -6331,7 +6331,7 @@
       <c r="I177" s="39"/>
       <c r="J177" s="32"/>
     </row>
-    <row r="178" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A178" s="26" t="s">
         <v>289</v>
       </c>
@@ -6351,55 +6351,55 @@
       <c r="I178" s="31"/>
       <c r="J178" s="32"/>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H179" s="99"/>
       <c r="I179" s="99"/>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H180" s="99"/>
       <c r="I180" s="99"/>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H181" s="99"/>
       <c r="I181" s="99"/>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H182" s="99"/>
       <c r="I182" s="99"/>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H183" s="99"/>
       <c r="I183" s="99"/>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H184" s="99"/>
       <c r="I184" s="99"/>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H185" s="99"/>
       <c r="I185" s="99"/>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H186" s="99"/>
       <c r="I186" s="99"/>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H187" s="99"/>
       <c r="I187" s="99"/>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H188" s="99"/>
       <c r="I188" s="99"/>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H189" s="99"/>
       <c r="I189" s="99"/>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H190" s="99"/>
       <c r="I190" s="99"/>
     </row>
-    <row r="210" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B210" s="100"/>
       <c r="C210" s="100"/>
       <c r="D210" s="100"/>
@@ -6410,7 +6410,7 @@
       <c r="I210" s="100"/>
       <c r="J210" s="100"/>
     </row>
-    <row r="211" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B211" s="100"/>
       <c r="C211" s="100"/>
       <c r="D211" s="100"/>
@@ -6421,7 +6421,7 @@
       <c r="I211" s="100"/>
       <c r="J211" s="100"/>
     </row>
-    <row r="212" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B212" s="100"/>
       <c r="C212" s="100"/>
       <c r="D212" s="100"/>
@@ -6432,7 +6432,7 @@
       <c r="I212" s="100"/>
       <c r="J212" s="100"/>
     </row>
-    <row r="213" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B213" s="100"/>
       <c r="C213" s="100"/>
       <c r="D213" s="100"/>
@@ -6443,7 +6443,7 @@
       <c r="I213" s="100"/>
       <c r="J213" s="100"/>
     </row>
-    <row r="214" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B214" s="100"/>
       <c r="C214" s="100"/>
       <c r="D214" s="100"/>
@@ -6454,7 +6454,7 @@
       <c r="I214" s="100"/>
       <c r="J214" s="100"/>
     </row>
-    <row r="215" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B215" s="100"/>
       <c r="C215" s="100"/>
       <c r="D215" s="100"/>
@@ -6465,7 +6465,7 @@
       <c r="I215" s="100"/>
       <c r="J215" s="100"/>
     </row>
-    <row r="216" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B216" s="100"/>
       <c r="C216" s="100"/>
       <c r="D216" s="100"/>
@@ -6476,7 +6476,7 @@
       <c r="I216" s="100"/>
       <c r="J216" s="100"/>
     </row>
-    <row r="217" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B217" s="100"/>
       <c r="C217" s="100"/>
       <c r="D217" s="100"/>
@@ -6487,7 +6487,7 @@
       <c r="I217" s="100"/>
       <c r="J217" s="100"/>
     </row>
-    <row r="218" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B218" s="100"/>
       <c r="C218" s="100"/>
       <c r="D218" s="100"/>
@@ -6498,7 +6498,7 @@
       <c r="I218" s="100"/>
       <c r="J218" s="100"/>
     </row>
-    <row r="219" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B219" s="100"/>
       <c r="C219" s="100"/>
       <c r="D219" s="100"/>
@@ -6509,7 +6509,7 @@
       <c r="I219" s="100"/>
       <c r="J219" s="100"/>
     </row>
-    <row r="220" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B220" s="100"/>
       <c r="C220" s="100"/>
       <c r="D220" s="100"/>
@@ -6520,7 +6520,7 @@
       <c r="I220" s="100"/>
       <c r="J220" s="100"/>
     </row>
-    <row r="221" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B221" s="100"/>
       <c r="C221" s="100"/>
       <c r="D221" s="100"/>
@@ -6531,7 +6531,7 @@
       <c r="I221" s="100"/>
       <c r="J221" s="100"/>
     </row>
-    <row r="222" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B222" s="100"/>
       <c r="C222" s="100"/>
       <c r="D222" s="100"/>
@@ -6542,7 +6542,7 @@
       <c r="I222" s="100"/>
       <c r="J222" s="100"/>
     </row>
-    <row r="223" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B223" s="100"/>
       <c r="C223" s="100"/>
       <c r="D223" s="100"/>
@@ -6553,7 +6553,7 @@
       <c r="I223" s="100"/>
       <c r="J223" s="100"/>
     </row>
-    <row r="224" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B224" s="100"/>
       <c r="C224" s="100"/>
       <c r="D224" s="100"/>
@@ -6564,7 +6564,7 @@
       <c r="I224" s="100"/>
       <c r="J224" s="100"/>
     </row>
-    <row r="225" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B225" s="100"/>
       <c r="C225" s="100"/>
       <c r="D225" s="100"/>
@@ -6575,7 +6575,7 @@
       <c r="I225" s="100"/>
       <c r="J225" s="100"/>
     </row>
-    <row r="226" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B226" s="100"/>
       <c r="C226" s="100"/>
       <c r="D226" s="100"/>
@@ -6586,7 +6586,7 @@
       <c r="I226" s="100"/>
       <c r="J226" s="100"/>
     </row>
-    <row r="227" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B227" s="100"/>
       <c r="C227" s="100"/>
       <c r="D227" s="100"/>
@@ -6597,7 +6597,7 @@
       <c r="I227" s="100"/>
       <c r="J227" s="100"/>
     </row>
-    <row r="228" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B228" s="100"/>
       <c r="C228" s="100"/>
       <c r="D228" s="100"/>
@@ -6608,7 +6608,7 @@
       <c r="I228" s="100"/>
       <c r="J228" s="100"/>
     </row>
-    <row r="229" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B229" s="100"/>
       <c r="C229" s="100"/>
       <c r="D229" s="100"/>
@@ -6619,7 +6619,7 @@
       <c r="I229" s="100"/>
       <c r="J229" s="100"/>
     </row>
-    <row r="230" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B230" s="100"/>
       <c r="C230" s="100"/>
       <c r="D230" s="100"/>
@@ -6630,7 +6630,7 @@
       <c r="I230" s="100"/>
       <c r="J230" s="100"/>
     </row>
-    <row r="231" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B231" s="100"/>
       <c r="C231" s="100"/>
       <c r="D231" s="100"/>
@@ -6641,7 +6641,7 @@
       <c r="I231" s="100"/>
       <c r="J231" s="100"/>
     </row>
-    <row r="232" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B232" s="100"/>
       <c r="C232" s="100"/>
       <c r="D232" s="100"/>
@@ -6652,7 +6652,7 @@
       <c r="I232" s="100"/>
       <c r="J232" s="100"/>
     </row>
-    <row r="233" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B233" s="100"/>
       <c r="C233" s="100"/>
       <c r="D233" s="100"/>
@@ -6663,7 +6663,7 @@
       <c r="I233" s="100"/>
       <c r="J233" s="100"/>
     </row>
-    <row r="234" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B234" s="100"/>
       <c r="C234" s="100"/>
       <c r="D234" s="100"/>
@@ -6674,7 +6674,7 @@
       <c r="I234" s="100"/>
       <c r="J234" s="100"/>
     </row>
-    <row r="235" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B235" s="100"/>
       <c r="C235" s="100"/>
       <c r="D235" s="100"/>
@@ -6685,7 +6685,7 @@
       <c r="I235" s="100"/>
       <c r="J235" s="100"/>
     </row>
-    <row r="236" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B236" s="100"/>
       <c r="C236" s="100"/>
       <c r="D236" s="100"/>
@@ -6696,7 +6696,7 @@
       <c r="I236" s="100"/>
       <c r="J236" s="100"/>
     </row>
-    <row r="237" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B237" s="100"/>
       <c r="C237" s="100"/>
       <c r="D237" s="100"/>
@@ -6707,7 +6707,7 @@
       <c r="I237" s="100"/>
       <c r="J237" s="100"/>
     </row>
-    <row r="238" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B238" s="100"/>
       <c r="C238" s="100"/>
       <c r="D238" s="100"/>
@@ -6718,7 +6718,7 @@
       <c r="I238" s="100"/>
       <c r="J238" s="100"/>
     </row>
-    <row r="239" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B239" s="100"/>
       <c r="C239" s="100"/>
       <c r="D239" s="100"/>
@@ -6729,7 +6729,7 @@
       <c r="I239" s="100"/>
       <c r="J239" s="100"/>
     </row>
-    <row r="240" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B240" s="100"/>
       <c r="C240" s="100"/>
       <c r="D240" s="100"/>
@@ -6740,7 +6740,7 @@
       <c r="I240" s="100"/>
       <c r="J240" s="100"/>
     </row>
-    <row r="241" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B241" s="100"/>
       <c r="C241" s="100"/>
       <c r="D241" s="100"/>
@@ -6751,7 +6751,7 @@
       <c r="I241" s="100"/>
       <c r="J241" s="100"/>
     </row>
-    <row r="242" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B242" s="100"/>
       <c r="C242" s="100"/>
       <c r="D242" s="100"/>
@@ -6762,7 +6762,7 @@
       <c r="I242" s="100"/>
       <c r="J242" s="100"/>
     </row>
-    <row r="243" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B243" s="100"/>
       <c r="C243" s="100"/>
       <c r="D243" s="100"/>
@@ -6773,7 +6773,7 @@
       <c r="I243" s="100"/>
       <c r="J243" s="100"/>
     </row>
-    <row r="244" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B244" s="100"/>
       <c r="C244" s="100"/>
       <c r="D244" s="100"/>
@@ -6784,7 +6784,7 @@
       <c r="I244" s="100"/>
       <c r="J244" s="100"/>
     </row>
-    <row r="245" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B245" s="100"/>
       <c r="C245" s="100"/>
       <c r="D245" s="100"/>
@@ -6795,7 +6795,7 @@
       <c r="I245" s="100"/>
       <c r="J245" s="100"/>
     </row>
-    <row r="246" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B246" s="100"/>
       <c r="C246" s="100"/>
       <c r="D246" s="100"/>
@@ -6806,7 +6806,7 @@
       <c r="I246" s="100"/>
       <c r="J246" s="100"/>
     </row>
-    <row r="247" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B247" s="100"/>
       <c r="C247" s="100"/>
       <c r="D247" s="100"/>
@@ -6817,7 +6817,7 @@
       <c r="I247" s="100"/>
       <c r="J247" s="100"/>
     </row>
-    <row r="248" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B248" s="100"/>
       <c r="C248" s="100"/>
       <c r="D248" s="100"/>
@@ -6828,7 +6828,7 @@
       <c r="I248" s="100"/>
       <c r="J248" s="100"/>
     </row>
-    <row r="249" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B249" s="100"/>
       <c r="C249" s="100"/>
       <c r="D249" s="100"/>
@@ -6839,7 +6839,7 @@
       <c r="I249" s="100"/>
       <c r="J249" s="100"/>
     </row>
-    <row r="250" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B250" s="100"/>
       <c r="C250" s="100"/>
       <c r="D250" s="100"/>
@@ -6850,7 +6850,7 @@
       <c r="I250" s="100"/>
       <c r="J250" s="100"/>
     </row>
-    <row r="251" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B251" s="100"/>
       <c r="C251" s="100"/>
       <c r="D251" s="100"/>
@@ -6861,7 +6861,7 @@
       <c r="I251" s="100"/>
       <c r="J251" s="100"/>
     </row>
-    <row r="252" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B252" s="100"/>
       <c r="C252" s="100"/>
       <c r="D252" s="100"/>
@@ -6872,7 +6872,7 @@
       <c r="I252" s="100"/>
       <c r="J252" s="100"/>
     </row>
-    <row r="253" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B253" s="100"/>
       <c r="C253" s="100"/>
       <c r="D253" s="100"/>
@@ -6883,7 +6883,7 @@
       <c r="I253" s="100"/>
       <c r="J253" s="100"/>
     </row>
-    <row r="254" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B254" s="100"/>
       <c r="C254" s="100"/>
       <c r="D254" s="100"/>
@@ -6894,7 +6894,7 @@
       <c r="I254" s="100"/>
       <c r="J254" s="100"/>
     </row>
-    <row r="255" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B255" s="100"/>
       <c r="C255" s="100"/>
       <c r="D255" s="100"/>
@@ -6905,7 +6905,7 @@
       <c r="I255" s="100"/>
       <c r="J255" s="100"/>
     </row>
-    <row r="256" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B256" s="100"/>
       <c r="C256" s="100"/>
       <c r="D256" s="100"/>
@@ -6916,7 +6916,7 @@
       <c r="I256" s="100"/>
       <c r="J256" s="100"/>
     </row>
-    <row r="257" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B257" s="100"/>
       <c r="C257" s="100"/>
       <c r="D257" s="100"/>
@@ -6927,7 +6927,7 @@
       <c r="I257" s="100"/>
       <c r="J257" s="100"/>
     </row>
-    <row r="258" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B258" s="100"/>
       <c r="C258" s="100"/>
       <c r="D258" s="100"/>
@@ -6938,7 +6938,7 @@
       <c r="I258" s="100"/>
       <c r="J258" s="100"/>
     </row>
-    <row r="259" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B259" s="100"/>
       <c r="C259" s="100"/>
       <c r="D259" s="100"/>
@@ -6949,7 +6949,7 @@
       <c r="I259" s="100"/>
       <c r="J259" s="100"/>
     </row>
-    <row r="260" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B260" s="100"/>
       <c r="C260" s="100"/>
       <c r="D260" s="100"/>
@@ -6960,7 +6960,7 @@
       <c r="I260" s="100"/>
       <c r="J260" s="100"/>
     </row>
-    <row r="261" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B261" s="100"/>
       <c r="C261" s="100"/>
       <c r="D261" s="100"/>
@@ -6971,7 +6971,7 @@
       <c r="I261" s="100"/>
       <c r="J261" s="100"/>
     </row>
-    <row r="262" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B262" s="100"/>
       <c r="C262" s="100"/>
       <c r="D262" s="100"/>
@@ -6982,7 +6982,7 @@
       <c r="I262" s="100"/>
       <c r="J262" s="100"/>
     </row>
-    <row r="263" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B263" s="100"/>
       <c r="C263" s="100"/>
       <c r="D263" s="100"/>
@@ -6993,7 +6993,7 @@
       <c r="I263" s="100"/>
       <c r="J263" s="100"/>
     </row>
-    <row r="264" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B264" s="100"/>
       <c r="C264" s="100"/>
       <c r="D264" s="100"/>
@@ -7004,7 +7004,7 @@
       <c r="I264" s="100"/>
       <c r="J264" s="100"/>
     </row>
-    <row r="265" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B265" s="100"/>
       <c r="C265" s="100"/>
       <c r="D265" s="100"/>
@@ -7015,7 +7015,7 @@
       <c r="I265" s="100"/>
       <c r="J265" s="100"/>
     </row>
-    <row r="266" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B266" s="100"/>
       <c r="C266" s="100"/>
       <c r="D266" s="100"/>
@@ -7026,7 +7026,7 @@
       <c r="I266" s="100"/>
       <c r="J266" s="100"/>
     </row>
-    <row r="267" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B267" s="100"/>
       <c r="C267" s="100"/>
       <c r="D267" s="100"/>
@@ -7037,7 +7037,7 @@
       <c r="I267" s="100"/>
       <c r="J267" s="100"/>
     </row>
-    <row r="268" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B268" s="100"/>
       <c r="C268" s="100"/>
       <c r="D268" s="100"/>
@@ -7048,7 +7048,7 @@
       <c r="I268" s="100"/>
       <c r="J268" s="100"/>
     </row>
-    <row r="269" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B269" s="100"/>
       <c r="C269" s="100"/>
       <c r="D269" s="100"/>
@@ -7059,651 +7059,656 @@
       <c r="I269" s="100"/>
       <c r="J269" s="100"/>
     </row>
-    <row r="270" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B270" s="100"/>
       <c r="G270" s="99"/>
     </row>
-    <row r="271" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B271" s="100"/>
       <c r="G271" s="99"/>
     </row>
-    <row r="272" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B272" s="100"/>
       <c r="G272" s="99"/>
     </row>
-    <row r="273" spans="2:7" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="2:7" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B273" s="100"/>
       <c r="G273" s="99"/>
     </row>
-    <row r="274" spans="2:7" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="2:7" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B274" s="100"/>
       <c r="G274" s="99"/>
     </row>
-    <row r="275" spans="2:7" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="2:7" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B275" s="100"/>
       <c r="G275" s="99"/>
     </row>
-    <row r="276" spans="2:7" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="2:7" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B276" s="100"/>
       <c r="G276" s="99"/>
     </row>
-    <row r="277" spans="2:7" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="2:7" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B277" s="100"/>
       <c r="G277" s="99"/>
     </row>
-    <row r="278" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B278" s="100"/>
       <c r="G278" s="99"/>
     </row>
-    <row r="279" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B279" s="100"/>
       <c r="G279" s="99"/>
     </row>
-    <row r="280" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B280" s="100"/>
       <c r="G280" s="99"/>
     </row>
-    <row r="281" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B281" s="100"/>
       <c r="G281" s="99"/>
     </row>
-    <row r="282" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B282" s="100"/>
       <c r="G282" s="99"/>
     </row>
-    <row r="283" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B283" s="100"/>
       <c r="G283" s="99"/>
     </row>
-    <row r="284" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B284" s="100"/>
       <c r="G284" s="99"/>
     </row>
-    <row r="285" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B285" s="100"/>
       <c r="G285" s="99"/>
     </row>
-    <row r="286" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B286" s="100"/>
       <c r="G286" s="99"/>
     </row>
-    <row r="287" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B287" s="100"/>
       <c r="G287" s="99"/>
     </row>
-    <row r="288" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B288" s="100"/>
       <c r="G288" s="99"/>
     </row>
-    <row r="289" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B289" s="100"/>
       <c r="G289" s="99"/>
     </row>
-    <row r="290" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B290" s="100"/>
       <c r="G290" s="99"/>
     </row>
-    <row r="291" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B291" s="100"/>
       <c r="G291" s="99"/>
     </row>
-    <row r="292" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B292" s="100"/>
       <c r="G292" s="99"/>
     </row>
-    <row r="293" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B293" s="100"/>
       <c r="G293" s="99"/>
     </row>
-    <row r="294" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B294" s="100"/>
       <c r="G294" s="99"/>
     </row>
-    <row r="295" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B295" s="100"/>
       <c r="G295" s="99"/>
     </row>
-    <row r="296" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B296" s="100"/>
       <c r="G296" s="99"/>
     </row>
-    <row r="297" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B297" s="100"/>
       <c r="G297" s="99"/>
     </row>
-    <row r="298" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B298" s="100"/>
       <c r="G298" s="99"/>
     </row>
-    <row r="299" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B299" s="100"/>
       <c r="G299" s="99"/>
     </row>
-    <row r="300" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B300" s="100"/>
       <c r="G300" s="99"/>
     </row>
-    <row r="301" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B301" s="100"/>
       <c r="G301" s="99"/>
     </row>
-    <row r="302" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B302" s="100"/>
       <c r="G302" s="99"/>
     </row>
-    <row r="303" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B303" s="100"/>
       <c r="G303" s="99"/>
     </row>
-    <row r="304" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B304" s="100"/>
       <c r="G304" s="99"/>
     </row>
-    <row r="305" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B305" s="100"/>
       <c r="G305" s="99"/>
     </row>
-    <row r="306" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B306" s="100"/>
       <c r="G306" s="99"/>
     </row>
-    <row r="307" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B307" s="100"/>
       <c r="G307" s="99"/>
     </row>
-    <row r="308" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B308" s="100"/>
       <c r="G308" s="99"/>
     </row>
-    <row r="309" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B309" s="100"/>
       <c r="G309" s="99"/>
     </row>
-    <row r="310" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B310" s="100"/>
       <c r="G310" s="99"/>
     </row>
-    <row r="311" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B311" s="100"/>
       <c r="G311" s="99"/>
     </row>
-    <row r="312" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B312" s="100"/>
       <c r="G312" s="99"/>
     </row>
-    <row r="313" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B313" s="100"/>
       <c r="G313" s="99"/>
     </row>
-    <row r="314" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B314" s="100"/>
       <c r="G314" s="99"/>
     </row>
-    <row r="315" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B315" s="100"/>
       <c r="G315" s="99"/>
     </row>
-    <row r="316" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B316" s="100"/>
       <c r="G316" s="99"/>
     </row>
-    <row r="317" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B317" s="100"/>
       <c r="G317" s="99"/>
     </row>
-    <row r="318" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B318" s="100"/>
       <c r="G318" s="99"/>
     </row>
-    <row r="319" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G319" s="99"/>
     </row>
-    <row r="320" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="2:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G320" s="99"/>
     </row>
-    <row r="321" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G321" s="99"/>
     </row>
-    <row r="322" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G322" s="99"/>
     </row>
-    <row r="323" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G323" s="99"/>
     </row>
-    <row r="324" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G324" s="99"/>
     </row>
-    <row r="325" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G325" s="99"/>
     </row>
-    <row r="326" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G326" s="99"/>
     </row>
-    <row r="327" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G327" s="99"/>
     </row>
-    <row r="328" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G328" s="99"/>
     </row>
-    <row r="329" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G329" s="99"/>
     </row>
-    <row r="330" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G330" s="99"/>
     </row>
-    <row r="331" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G331" s="99"/>
     </row>
-    <row r="332" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G332" s="99"/>
     </row>
-    <row r="333" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G333" s="99"/>
     </row>
-    <row r="334" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G334" s="99"/>
     </row>
-    <row r="335" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G335" s="99"/>
     </row>
-    <row r="336" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G336" s="99"/>
     </row>
-    <row r="337" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G337" s="99"/>
     </row>
-    <row r="338" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G338" s="99"/>
     </row>
-    <row r="339" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G339" s="99"/>
     </row>
-    <row r="340" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G340" s="99"/>
     </row>
-    <row r="341" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="341" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G341" s="99"/>
     </row>
-    <row r="342" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G342" s="99"/>
     </row>
-    <row r="343" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G343" s="99"/>
     </row>
-    <row r="344" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G344" s="99"/>
     </row>
-    <row r="345" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="345" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G345" s="99"/>
     </row>
-    <row r="346" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G346" s="99"/>
     </row>
-    <row r="347" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G347" s="99"/>
     </row>
-    <row r="348" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G348" s="99"/>
     </row>
-    <row r="349" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="349" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G349" s="99"/>
     </row>
-    <row r="350" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="350" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G350" s="99"/>
     </row>
-    <row r="351" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="351" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G351" s="99"/>
     </row>
-    <row r="352" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="352" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G352" s="99"/>
     </row>
-    <row r="353" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="353" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G353" s="99"/>
     </row>
-    <row r="354" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="354" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G354" s="99"/>
     </row>
-    <row r="355" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="355" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G355" s="99"/>
     </row>
-    <row r="356" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G356" s="99"/>
     </row>
-    <row r="357" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G357" s="99"/>
     </row>
-    <row r="358" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G358" s="99"/>
     </row>
-    <row r="359" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="359" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G359" s="99"/>
     </row>
-    <row r="360" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="360" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G360" s="99"/>
     </row>
-    <row r="361" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="361" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G361" s="99"/>
     </row>
-    <row r="362" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="362" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G362" s="99"/>
     </row>
-    <row r="363" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="363" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G363" s="99"/>
     </row>
-    <row r="364" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G364" s="99"/>
     </row>
-    <row r="365" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G365" s="99"/>
     </row>
-    <row r="366" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G366" s="99"/>
     </row>
-    <row r="367" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G367" s="99"/>
     </row>
-    <row r="368" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="368" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G368" s="99"/>
     </row>
-    <row r="369" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G369" s="99"/>
     </row>
-    <row r="370" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="370" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G370" s="99"/>
     </row>
-    <row r="371" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G371" s="99"/>
     </row>
-    <row r="372" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G372" s="99"/>
     </row>
-    <row r="373" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G373" s="99"/>
     </row>
-    <row r="374" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="374" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G374" s="99"/>
     </row>
-    <row r="375" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="375" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G375" s="99"/>
     </row>
-    <row r="376" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G376" s="99"/>
     </row>
-    <row r="377" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="377" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G377" s="99"/>
     </row>
-    <row r="378" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="378" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G378" s="99"/>
     </row>
-    <row r="379" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="379" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G379" s="99"/>
     </row>
-    <row r="380" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="380" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G380" s="99"/>
     </row>
-    <row r="381" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="381" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G381" s="99"/>
     </row>
-    <row r="382" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G382" s="99"/>
     </row>
-    <row r="383" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="383" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G383" s="99"/>
     </row>
-    <row r="384" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="384" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G384" s="99"/>
     </row>
-    <row r="385" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="385" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G385" s="99"/>
     </row>
-    <row r="386" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="386" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G386" s="99"/>
     </row>
-    <row r="387" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="387" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G387" s="99"/>
     </row>
-    <row r="388" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="388" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G388" s="99"/>
     </row>
-    <row r="389" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="389" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G389" s="99"/>
     </row>
-    <row r="390" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="390" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G390" s="99"/>
     </row>
-    <row r="391" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="391" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G391" s="99"/>
     </row>
-    <row r="392" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="392" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G392" s="99"/>
     </row>
-    <row r="393" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="393" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G393" s="99"/>
     </row>
-    <row r="394" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="394" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G394" s="99"/>
     </row>
-    <row r="395" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="395" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G395" s="99"/>
     </row>
-    <row r="396" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="396" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G396" s="99"/>
     </row>
-    <row r="397" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="397" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G397" s="99"/>
     </row>
-    <row r="398" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="398" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G398" s="99"/>
     </row>
-    <row r="399" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="399" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G399" s="99"/>
     </row>
-    <row r="400" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="400" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G400" s="99"/>
     </row>
-    <row r="401" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="401" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G401" s="99"/>
     </row>
-    <row r="402" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="402" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G402" s="99"/>
     </row>
-    <row r="403" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="403" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G403" s="99"/>
     </row>
-    <row r="404" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="404" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G404" s="99"/>
     </row>
-    <row r="405" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="405" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G405" s="99"/>
     </row>
-    <row r="406" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="406" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G406" s="99"/>
     </row>
-    <row r="407" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="407" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G407" s="99"/>
     </row>
-    <row r="408" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="408" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G408" s="99"/>
     </row>
-    <row r="409" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="409" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G409" s="99"/>
     </row>
-    <row r="410" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="410" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G410" s="99"/>
     </row>
-    <row r="411" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="411" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G411" s="99"/>
     </row>
-    <row r="412" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="412" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G412" s="99"/>
     </row>
-    <row r="413" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="413" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G413" s="99"/>
     </row>
-    <row r="414" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="414" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G414" s="99"/>
     </row>
-    <row r="415" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="415" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G415" s="99"/>
     </row>
-    <row r="416" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="416" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G416" s="99"/>
     </row>
-    <row r="417" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="417" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G417" s="99"/>
     </row>
-    <row r="418" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="418" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G418" s="99"/>
     </row>
-    <row r="419" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="419" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G419" s="99"/>
     </row>
-    <row r="420" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="420" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G420" s="99"/>
     </row>
-    <row r="421" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="421" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G421" s="99"/>
     </row>
-    <row r="422" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="422" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G422" s="99"/>
     </row>
-    <row r="423" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="423" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G423" s="99"/>
     </row>
-    <row r="424" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="424" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G424" s="99"/>
     </row>
-    <row r="425" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="425" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G425" s="99"/>
     </row>
-    <row r="426" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="426" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G426" s="99"/>
     </row>
-    <row r="427" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="427" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G427" s="99"/>
     </row>
-    <row r="428" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="428" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G428" s="99"/>
     </row>
-    <row r="429" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="429" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G429" s="99"/>
     </row>
-    <row r="430" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="430" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G430" s="99"/>
     </row>
-    <row r="431" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="431" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G431" s="99"/>
     </row>
-    <row r="432" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="432" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G432" s="99"/>
     </row>
-    <row r="433" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="433" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G433" s="99"/>
     </row>
-    <row r="434" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="434" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G434" s="99"/>
     </row>
-    <row r="435" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="435" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G435" s="99"/>
     </row>
-    <row r="436" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="436" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G436" s="99"/>
     </row>
-    <row r="437" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="437" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G437" s="99"/>
     </row>
-    <row r="438" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="438" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G438" s="99"/>
     </row>
-    <row r="439" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="439" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G439" s="99"/>
     </row>
-    <row r="440" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="440" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G440" s="99"/>
     </row>
-    <row r="441" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="441" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G441" s="99"/>
     </row>
-    <row r="442" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="442" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G442" s="99"/>
     </row>
-    <row r="443" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="443" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G443" s="99"/>
     </row>
-    <row r="444" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="444" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G444" s="99"/>
     </row>
-    <row r="445" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="445" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G445" s="99"/>
     </row>
-    <row r="446" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="446" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G446" s="99"/>
     </row>
-    <row r="447" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="447" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G447" s="99"/>
     </row>
-    <row r="448" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="448" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G448" s="99"/>
     </row>
-    <row r="449" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="449" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G449" s="99"/>
     </row>
-    <row r="450" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="450" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G450" s="99"/>
     </row>
-    <row r="451" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="451" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G451" s="99"/>
     </row>
-    <row r="452" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="452" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G452" s="99"/>
     </row>
-    <row r="453" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="453" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G453" s="99"/>
     </row>
-    <row r="454" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="454" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G454" s="99"/>
     </row>
-    <row r="455" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="455" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G455" s="99"/>
     </row>
-    <row r="456" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="456" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G456" s="99"/>
     </row>
-    <row r="457" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="457" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G457" s="99"/>
     </row>
-    <row r="458" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="458" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G458" s="99"/>
     </row>
-    <row r="459" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="459" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G459" s="99"/>
     </row>
-    <row r="460" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="460" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G460" s="99"/>
     </row>
-    <row r="461" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="461" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G461" s="99"/>
     </row>
-    <row r="462" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="462" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G462" s="99"/>
     </row>
-    <row r="463" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="463" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G463" s="99"/>
     </row>
-    <row r="464" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="464" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G464" s="99"/>
     </row>
-    <row r="465" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="465" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G465" s="99"/>
     </row>
-    <row r="466" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="466" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G466" s="99"/>
     </row>
-    <row r="467" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="467" spans="7:7" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="G467" s="99"/>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="K13:K14"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="A15:J15"/>
+    <mergeCell ref="A61:J61"/>
     <mergeCell ref="B6:H6"/>
     <mergeCell ref="B7:I7"/>
     <mergeCell ref="B9:I9"/>
@@ -7712,11 +7717,6 @@
     <mergeCell ref="C13:C14"/>
     <mergeCell ref="D13:F13"/>
     <mergeCell ref="G13:H13"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="K13:K14"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="A15:J15"/>
-    <mergeCell ref="A61:J61"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7725,43 +7725,43 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68E7129F-4618-4610-B852-D700608599C6}">
   <dimension ref="A1:K291"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="36.85546875" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" customWidth="1"/>
-    <col min="6" max="6" width="3.42578125" customWidth="1"/>
-    <col min="7" max="7" width="14.140625" customWidth="1"/>
-    <col min="8" max="8" width="2.7109375" customWidth="1"/>
-    <col min="9" max="9" width="2.5703125" customWidth="1"/>
-    <col min="10" max="10" width="23.5703125" customWidth="1"/>
+    <col min="1" max="1" width="36.81640625" customWidth="1"/>
+    <col min="2" max="2" width="22.453125" customWidth="1"/>
+    <col min="3" max="3" width="4.7265625" customWidth="1"/>
+    <col min="4" max="4" width="13.81640625" customWidth="1"/>
+    <col min="5" max="5" width="15.453125" customWidth="1"/>
+    <col min="6" max="6" width="3.453125" customWidth="1"/>
+    <col min="7" max="7" width="14.1796875" customWidth="1"/>
+    <col min="8" max="8" width="2.7265625" customWidth="1"/>
+    <col min="9" max="9" width="2.54296875" customWidth="1"/>
+    <col min="10" max="10" width="23.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="164" t="s">
-        <v>346</v>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" s="140" t="s">
+        <v>344</v>
       </c>
       <c r="G1" s="1"/>
       <c r="I1" s="2"/>
       <c r="J1" s="3"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="165" t="s">
-        <v>347</v>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="141" t="s">
+        <v>345</v>
       </c>
       <c r="G2" s="1"/>
       <c r="I2" s="4"/>
       <c r="J2" s="5"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="G3" s="1"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="5"/>
     </row>
-    <row r="4" spans="1:11" s="25" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" s="25" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="102" t="s">
         <v>83</v>
       </c>
@@ -7775,7 +7775,7 @@
       <c r="I4" s="102"/>
       <c r="J4" s="102"/>
     </row>
-    <row r="5" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="103" t="s">
         <v>291</v>
       </c>
@@ -7789,7 +7789,7 @@
       <c r="I5" s="104"/>
       <c r="J5" s="104"/>
     </row>
-    <row r="6" spans="1:11" s="35" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" s="35" customFormat="1" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="105"/>
       <c r="C6" s="100"/>
       <c r="D6" s="100"/>
@@ -7800,7 +7800,7 @@
       <c r="I6" s="100"/>
       <c r="J6" s="100"/>
     </row>
-    <row r="7" spans="1:11" s="25" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" s="25" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="106" t="s">
         <v>292</v>
       </c>
@@ -7814,7 +7814,7 @@
       <c r="I7" s="109"/>
       <c r="J7" s="109"/>
     </row>
-    <row r="8" spans="1:11" s="25" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" s="25" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="45" t="s">
         <v>293</v>
       </c>
@@ -7836,7 +7836,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="9" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="103" t="s">
         <v>298</v>
       </c>
@@ -7858,7 +7858,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="10" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="103" t="s">
         <v>302</v>
       </c>
@@ -7880,7 +7880,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="11" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="103" t="s">
         <v>303</v>
       </c>
@@ -7898,7 +7898,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="12" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="112" t="s">
         <v>304</v>
       </c>
@@ -7916,7 +7916,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="13" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="103" t="s">
         <v>306</v>
       </c>
@@ -7934,7 +7934,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="14" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="103" t="s">
         <v>307</v>
       </c>
@@ -7952,25 +7952,25 @@
         <v>301</v>
       </c>
     </row>
-    <row r="15" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="103" t="s">
         <v>308</v>
       </c>
       <c r="B15" s="111"/>
       <c r="C15" s="112"/>
       <c r="D15" s="112"/>
-      <c r="E15" s="157" t="s">
+      <c r="E15" s="163" t="s">
         <v>309</v>
       </c>
-      <c r="F15" s="157"/>
-      <c r="G15" s="157"/>
+      <c r="F15" s="163"/>
+      <c r="G15" s="163"/>
       <c r="H15" s="115"/>
       <c r="I15" s="112"/>
       <c r="J15" s="112" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="16" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="103" t="s">
         <v>310</v>
       </c>
@@ -7988,7 +7988,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="17" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="103" t="s">
         <v>311</v>
       </c>
@@ -8008,7 +8008,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="18" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="103"/>
       <c r="B18" s="111"/>
       <c r="C18" s="104"/>
@@ -8022,7 +8022,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="19" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="112" t="s">
         <v>315</v>
       </c>
@@ -8040,7 +8040,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="20" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="112" t="s">
         <v>316</v>
       </c>
@@ -8058,7 +8058,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="21" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="116" t="s">
         <v>317</v>
       </c>
@@ -8076,7 +8076,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="22" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" s="35" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="116" t="s">
         <v>318</v>
       </c>
@@ -8094,7 +8094,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="23" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="116" t="s">
         <v>319</v>
       </c>
@@ -8108,7 +8108,7 @@
       <c r="I23" s="118"/>
       <c r="J23" s="116"/>
     </row>
-    <row r="24" spans="1:10" s="125" customFormat="1" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" s="125" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="122" t="s">
         <v>320</v>
       </c>
@@ -8124,7 +8124,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="25" spans="1:10" s="35" customFormat="1" ht="12.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" s="35" customFormat="1" ht="12.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B25" s="105"/>
       <c r="C25" s="100"/>
       <c r="D25" s="100"/>
@@ -8135,7 +8135,7 @@
       <c r="I25" s="100"/>
       <c r="J25" s="100"/>
     </row>
-    <row r="26" spans="1:10" s="25" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" s="25" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="45" t="s">
         <v>321</v>
       </c>
@@ -8160,41 +8160,41 @@
       <c r="I27" s="100"/>
       <c r="J27" s="100"/>
     </row>
-    <row r="28" spans="1:10" s="33" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="158" t="s">
+    <row r="28" spans="1:10" s="33" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="164" t="s">
         <v>322</v>
       </c>
-      <c r="B28" s="158"/>
+      <c r="B28" s="164"/>
       <c r="C28" s="72"/>
-      <c r="D28" s="159"/>
-      <c r="E28" s="160"/>
-      <c r="F28" s="160"/>
-      <c r="G28" s="161"/>
+      <c r="D28" s="165"/>
+      <c r="E28" s="166"/>
+      <c r="F28" s="166"/>
+      <c r="G28" s="167"/>
       <c r="H28" s="112"/>
       <c r="I28" s="127"/>
       <c r="J28" s="128" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="29" spans="1:10" s="33" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="158" t="s">
+    <row r="29" spans="1:10" s="33" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="164" t="s">
         <v>324</v>
       </c>
-      <c r="B29" s="158"/>
+      <c r="B29" s="164"/>
       <c r="C29" s="129"/>
-      <c r="D29" s="162" t="s">
+      <c r="D29" s="168" t="s">
         <v>325</v>
       </c>
-      <c r="E29" s="162"/>
-      <c r="F29" s="162"/>
-      <c r="G29" s="163"/>
+      <c r="E29" s="168"/>
+      <c r="F29" s="168"/>
+      <c r="G29" s="169"/>
       <c r="H29" s="112"/>
       <c r="I29" s="26"/>
       <c r="J29" s="128" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="30" spans="1:10" s="35" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" s="35" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="130" t="s">
         <v>327</v>
       </c>
@@ -8212,7 +8212,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="31" spans="1:10" s="35" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" s="35" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="130" t="s">
         <v>330</v>
       </c>
@@ -8230,7 +8230,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="32" spans="1:10" s="35" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" s="35" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="100"/>
       <c r="C32" s="100"/>
       <c r="D32" s="100"/>
@@ -8241,7 +8241,7 @@
       <c r="I32" s="100"/>
       <c r="J32" s="100"/>
     </row>
-    <row r="33" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="133" t="s">
         <v>332</v>
       </c>
@@ -8255,7 +8255,7 @@
       <c r="I33" s="134"/>
       <c r="J33" s="134"/>
     </row>
-    <row r="34" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="135" t="s">
         <v>333</v>
       </c>
@@ -8273,7 +8273,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="35" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="136" t="s">
         <v>324</v>
       </c>
@@ -8291,7 +8291,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="36" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="136" t="s">
         <v>327</v>
       </c>
@@ -8309,7 +8309,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="37" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="136" t="s">
         <v>338</v>
       </c>
@@ -8327,7 +8327,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="38" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="119"/>
       <c r="B38" s="118"/>
       <c r="C38" s="100"/>
@@ -8339,7 +8339,7 @@
       <c r="I38" s="100"/>
       <c r="J38" s="100"/>
     </row>
-    <row r="39" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="100"/>
       <c r="C39" s="100"/>
       <c r="D39" s="100"/>
@@ -8350,7 +8350,7 @@
       <c r="I39" s="100"/>
       <c r="J39" s="100"/>
     </row>
-    <row r="40" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="100"/>
       <c r="C40" s="100"/>
       <c r="D40" s="100"/>
@@ -8361,7 +8361,7 @@
       <c r="I40" s="100"/>
       <c r="J40" s="100"/>
     </row>
-    <row r="41" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="100"/>
       <c r="C41" s="100"/>
       <c r="D41" s="100"/>
@@ -8372,7 +8372,7 @@
       <c r="I41" s="100"/>
       <c r="J41" s="100"/>
     </row>
-    <row r="42" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="100"/>
       <c r="C42" s="100"/>
       <c r="D42" s="100"/>
@@ -8383,7 +8383,7 @@
       <c r="I42" s="100"/>
       <c r="J42" s="100"/>
     </row>
-    <row r="43" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B43" s="100"/>
       <c r="C43" s="100"/>
       <c r="D43" s="100"/>
@@ -8394,7 +8394,7 @@
       <c r="I43" s="100"/>
       <c r="J43" s="100"/>
     </row>
-    <row r="44" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B44" s="100"/>
       <c r="C44" s="100"/>
       <c r="D44" s="100"/>
@@ -8405,7 +8405,7 @@
       <c r="I44" s="100"/>
       <c r="J44" s="100"/>
     </row>
-    <row r="45" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B45" s="100"/>
       <c r="C45" s="100"/>
       <c r="D45" s="100"/>
@@ -8416,7 +8416,7 @@
       <c r="I45" s="100"/>
       <c r="J45" s="100"/>
     </row>
-    <row r="46" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B46" s="100"/>
       <c r="C46" s="100"/>
       <c r="D46" s="100"/>
@@ -8427,7 +8427,7 @@
       <c r="I46" s="100"/>
       <c r="J46" s="100"/>
     </row>
-    <row r="47" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B47" s="100"/>
       <c r="C47" s="100"/>
       <c r="D47" s="100"/>
@@ -8438,7 +8438,7 @@
       <c r="I47" s="100"/>
       <c r="J47" s="100"/>
     </row>
-    <row r="48" spans="1:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B48" s="100"/>
       <c r="C48" s="100" t="s">
         <v>83</v>
@@ -8451,7 +8451,7 @@
       <c r="I48" s="100"/>
       <c r="J48" s="100"/>
     </row>
-    <row r="49" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B49" s="100"/>
       <c r="C49" s="100"/>
       <c r="D49" s="100"/>
@@ -8462,7 +8462,7 @@
       <c r="I49" s="100"/>
       <c r="J49" s="100"/>
     </row>
-    <row r="50" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B50" s="100"/>
       <c r="C50" s="100"/>
       <c r="D50" s="100"/>
@@ -8473,7 +8473,7 @@
       <c r="I50" s="100"/>
       <c r="J50" s="100"/>
     </row>
-    <row r="51" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B51" s="100"/>
       <c r="C51" s="100"/>
       <c r="D51" s="100"/>
@@ -8484,7 +8484,7 @@
       <c r="I51" s="100"/>
       <c r="J51" s="100"/>
     </row>
-    <row r="52" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B52" s="100"/>
       <c r="C52" s="100"/>
       <c r="D52" s="100"/>
@@ -8495,7 +8495,7 @@
       <c r="I52" s="100"/>
       <c r="J52" s="100"/>
     </row>
-    <row r="53" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B53" s="100"/>
       <c r="C53" s="100"/>
       <c r="D53" s="100"/>
@@ -8506,7 +8506,7 @@
       <c r="I53" s="100"/>
       <c r="J53" s="100"/>
     </row>
-    <row r="54" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B54" s="100"/>
       <c r="C54" s="100"/>
       <c r="D54" s="100"/>
@@ -8517,7 +8517,7 @@
       <c r="I54" s="100"/>
       <c r="J54" s="100"/>
     </row>
-    <row r="55" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B55" s="100"/>
       <c r="C55" s="100"/>
       <c r="D55" s="100"/>
@@ -8528,7 +8528,7 @@
       <c r="I55" s="100"/>
       <c r="J55" s="100"/>
     </row>
-    <row r="56" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B56" s="100"/>
       <c r="C56" s="100"/>
       <c r="D56" s="100"/>
@@ -8539,7 +8539,7 @@
       <c r="I56" s="100"/>
       <c r="J56" s="100"/>
     </row>
-    <row r="57" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B57" s="100"/>
       <c r="C57" s="100"/>
       <c r="D57" s="100"/>
@@ -8550,7 +8550,7 @@
       <c r="I57" s="100"/>
       <c r="J57" s="100"/>
     </row>
-    <row r="58" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B58" s="100"/>
       <c r="C58" s="100"/>
       <c r="D58" s="100"/>
@@ -8561,7 +8561,7 @@
       <c r="I58" s="100"/>
       <c r="J58" s="100"/>
     </row>
-    <row r="59" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B59" s="100"/>
       <c r="C59" s="100"/>
       <c r="D59" s="100"/>
@@ -8572,7 +8572,7 @@
       <c r="I59" s="100"/>
       <c r="J59" s="100"/>
     </row>
-    <row r="60" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B60" s="100"/>
       <c r="C60" s="100"/>
       <c r="D60" s="100"/>
@@ -8583,7 +8583,7 @@
       <c r="I60" s="100"/>
       <c r="J60" s="100"/>
     </row>
-    <row r="61" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B61" s="100"/>
       <c r="C61" s="100" t="s">
         <v>340</v>
@@ -8596,7 +8596,7 @@
       <c r="I61" s="100"/>
       <c r="J61" s="100"/>
     </row>
-    <row r="62" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B62" s="100"/>
       <c r="C62" s="100"/>
       <c r="D62" s="100"/>
@@ -8607,7 +8607,7 @@
       <c r="I62" s="100"/>
       <c r="J62" s="100"/>
     </row>
-    <row r="63" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B63" s="100"/>
       <c r="C63" s="100"/>
       <c r="D63" s="100"/>
@@ -8618,7 +8618,7 @@
       <c r="I63" s="100"/>
       <c r="J63" s="100"/>
     </row>
-    <row r="64" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B64" s="100"/>
       <c r="C64" s="100"/>
       <c r="D64" s="100"/>
@@ -8629,7 +8629,7 @@
       <c r="I64" s="100"/>
       <c r="J64" s="100"/>
     </row>
-    <row r="65" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B65" s="100"/>
       <c r="C65" s="100"/>
       <c r="D65" s="100"/>
@@ -8640,7 +8640,7 @@
       <c r="I65" s="100"/>
       <c r="J65" s="100"/>
     </row>
-    <row r="66" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B66" s="100"/>
       <c r="C66" s="100"/>
       <c r="D66" s="100"/>
@@ -8651,7 +8651,7 @@
       <c r="I66" s="100"/>
       <c r="J66" s="100"/>
     </row>
-    <row r="67" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B67" s="100"/>
       <c r="C67" s="100"/>
       <c r="D67" s="100"/>
@@ -8662,7 +8662,7 @@
       <c r="I67" s="100"/>
       <c r="J67" s="100"/>
     </row>
-    <row r="68" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B68" s="100"/>
       <c r="C68" s="100"/>
       <c r="D68" s="100"/>
@@ -8673,7 +8673,7 @@
       <c r="I68" s="100"/>
       <c r="J68" s="100"/>
     </row>
-    <row r="69" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B69" s="100"/>
       <c r="C69" s="100"/>
       <c r="D69" s="100"/>
@@ -8684,7 +8684,7 @@
       <c r="I69" s="100"/>
       <c r="J69" s="100"/>
     </row>
-    <row r="70" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B70" s="100"/>
       <c r="C70" s="100"/>
       <c r="D70" s="100"/>
@@ -8695,7 +8695,7 @@
       <c r="I70" s="100"/>
       <c r="J70" s="100"/>
     </row>
-    <row r="71" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B71" s="100"/>
       <c r="C71" s="100"/>
       <c r="D71" s="100"/>
@@ -8706,7 +8706,7 @@
       <c r="I71" s="100"/>
       <c r="J71" s="100"/>
     </row>
-    <row r="72" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B72" s="100"/>
       <c r="C72" s="100"/>
       <c r="D72" s="100"/>
@@ -8717,7 +8717,7 @@
       <c r="I72" s="100"/>
       <c r="J72" s="100"/>
     </row>
-    <row r="73" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B73" s="100"/>
       <c r="C73" s="100"/>
       <c r="D73" s="100"/>
@@ -8728,7 +8728,7 @@
       <c r="I73" s="100"/>
       <c r="J73" s="100"/>
     </row>
-    <row r="74" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B74" s="100"/>
       <c r="C74" s="100"/>
       <c r="D74" s="100"/>
@@ -8739,7 +8739,7 @@
       <c r="I74" s="100"/>
       <c r="J74" s="100"/>
     </row>
-    <row r="75" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B75" s="100"/>
       <c r="C75" s="100"/>
       <c r="D75" s="100"/>
@@ -8750,7 +8750,7 @@
       <c r="I75" s="100"/>
       <c r="J75" s="100"/>
     </row>
-    <row r="76" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B76" s="100"/>
       <c r="C76" s="100"/>
       <c r="D76" s="100"/>
@@ -8761,7 +8761,7 @@
       <c r="I76" s="100"/>
       <c r="J76" s="100"/>
     </row>
-    <row r="77" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B77" s="100"/>
       <c r="C77" s="100"/>
       <c r="D77" s="100"/>
@@ -8772,7 +8772,7 @@
       <c r="I77" s="100"/>
       <c r="J77" s="100"/>
     </row>
-    <row r="78" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B78" s="100"/>
       <c r="C78" s="100"/>
       <c r="D78" s="100"/>
@@ -8783,7 +8783,7 @@
       <c r="I78" s="100"/>
       <c r="J78" s="100"/>
     </row>
-    <row r="79" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B79" s="100"/>
       <c r="C79" s="100"/>
       <c r="D79" s="100"/>
@@ -8794,7 +8794,7 @@
       <c r="I79" s="100"/>
       <c r="J79" s="100"/>
     </row>
-    <row r="80" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B80" s="100"/>
       <c r="C80" s="100"/>
       <c r="D80" s="100"/>
@@ -8805,7 +8805,7 @@
       <c r="I80" s="100"/>
       <c r="J80" s="100"/>
     </row>
-    <row r="81" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B81" s="100"/>
       <c r="C81" s="100"/>
       <c r="D81" s="100"/>
@@ -8816,7 +8816,7 @@
       <c r="I81" s="100"/>
       <c r="J81" s="100"/>
     </row>
-    <row r="82" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B82" s="100"/>
       <c r="C82" s="100"/>
       <c r="D82" s="100"/>
@@ -8827,7 +8827,7 @@
       <c r="I82" s="100"/>
       <c r="J82" s="100"/>
     </row>
-    <row r="83" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B83" s="100"/>
       <c r="C83" s="100"/>
       <c r="D83" s="100"/>
@@ -8838,7 +8838,7 @@
       <c r="I83" s="100"/>
       <c r="J83" s="100"/>
     </row>
-    <row r="84" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B84" s="100"/>
       <c r="C84" s="100"/>
       <c r="D84" s="100"/>
@@ -8849,7 +8849,7 @@
       <c r="I84" s="100"/>
       <c r="J84" s="100"/>
     </row>
-    <row r="85" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B85" s="100"/>
       <c r="C85" s="100"/>
       <c r="D85" s="100"/>
@@ -8860,7 +8860,7 @@
       <c r="I85" s="100"/>
       <c r="J85" s="100"/>
     </row>
-    <row r="86" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B86" s="100"/>
       <c r="C86" s="100"/>
       <c r="D86" s="100"/>
@@ -8871,7 +8871,7 @@
       <c r="I86" s="100"/>
       <c r="J86" s="100"/>
     </row>
-    <row r="87" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B87" s="100"/>
       <c r="C87" s="100"/>
       <c r="D87" s="100"/>
@@ -8882,7 +8882,7 @@
       <c r="I87" s="100"/>
       <c r="J87" s="100"/>
     </row>
-    <row r="88" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B88" s="100"/>
       <c r="C88" s="100"/>
       <c r="D88" s="100"/>
@@ -8893,7 +8893,7 @@
       <c r="I88" s="100"/>
       <c r="J88" s="100"/>
     </row>
-    <row r="89" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B89" s="100"/>
       <c r="C89" s="100"/>
       <c r="D89" s="100"/>
@@ -8904,7 +8904,7 @@
       <c r="I89" s="100"/>
       <c r="J89" s="100"/>
     </row>
-    <row r="90" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B90" s="100"/>
       <c r="C90" s="100"/>
       <c r="D90" s="100"/>
@@ -8915,7 +8915,7 @@
       <c r="I90" s="100"/>
       <c r="J90" s="100"/>
     </row>
-    <row r="91" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B91" s="100"/>
       <c r="C91" s="100"/>
       <c r="D91" s="100"/>
@@ -8926,7 +8926,7 @@
       <c r="I91" s="100"/>
       <c r="J91" s="100"/>
     </row>
-    <row r="92" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B92" s="100"/>
       <c r="C92" s="100"/>
       <c r="D92" s="100"/>
@@ -8937,7 +8937,7 @@
       <c r="I92" s="100"/>
       <c r="J92" s="100"/>
     </row>
-    <row r="93" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B93" s="100"/>
       <c r="C93" s="100"/>
       <c r="D93" s="100"/>
@@ -8948,204 +8948,204 @@
       <c r="I93" s="100"/>
       <c r="J93" s="100"/>
     </row>
-    <row r="94" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B94" s="100"/>
     </row>
-    <row r="95" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B95" s="100"/>
     </row>
-    <row r="96" spans="2:10" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:10" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B96" s="100"/>
     </row>
-    <row r="97" spans="2:2" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:2" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B97" s="100"/>
     </row>
-    <row r="98" spans="2:2" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:2" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B98" s="100"/>
     </row>
-    <row r="99" spans="2:2" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:2" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B99" s="100"/>
     </row>
-    <row r="100" spans="2:2" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:2" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B100" s="100"/>
     </row>
-    <row r="101" spans="2:2" s="35" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:2" s="35" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B101" s="100"/>
     </row>
-    <row r="102" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B102" s="100"/>
     </row>
-    <row r="103" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B103" s="100"/>
     </row>
-    <row r="104" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B104" s="100"/>
     </row>
-    <row r="105" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B105" s="100"/>
     </row>
-    <row r="106" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B106" s="100"/>
     </row>
-    <row r="107" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B107" s="100"/>
     </row>
-    <row r="108" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B108" s="100"/>
     </row>
-    <row r="109" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B109" s="100"/>
     </row>
-    <row r="110" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B110" s="100"/>
     </row>
-    <row r="111" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B111" s="100"/>
     </row>
-    <row r="112" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B112" s="100"/>
     </row>
-    <row r="113" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B113" s="100"/>
     </row>
-    <row r="114" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B114" s="100"/>
     </row>
-    <row r="115" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B115" s="100"/>
     </row>
-    <row r="116" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B116" s="100"/>
     </row>
-    <row r="117" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B117" s="100"/>
     </row>
-    <row r="118" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B118" s="100"/>
     </row>
-    <row r="119" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B119" s="100"/>
       <c r="J119" s="138" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="120" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B120" s="100"/>
     </row>
-    <row r="121" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B121" s="100"/>
     </row>
-    <row r="122" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B122" s="100"/>
     </row>
-    <row r="123" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B123" s="100"/>
     </row>
-    <row r="124" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B124" s="100"/>
     </row>
-    <row r="125" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B125" s="100"/>
     </row>
-    <row r="126" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B126" s="100"/>
     </row>
-    <row r="127" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B127" s="100"/>
     </row>
-    <row r="128" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:10" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B128" s="100"/>
     </row>
-    <row r="129" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B129" s="100"/>
     </row>
-    <row r="130" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B130" s="100"/>
     </row>
-    <row r="131" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B131" s="100"/>
     </row>
-    <row r="132" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B132" s="100"/>
     </row>
-    <row r="133" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B133" s="100"/>
     </row>
-    <row r="134" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B134" s="100"/>
     </row>
-    <row r="135" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B135" s="100"/>
     </row>
-    <row r="136" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B136" s="100"/>
     </row>
-    <row r="137" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B137" s="100"/>
     </row>
-    <row r="138" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B138" s="100"/>
     </row>
-    <row r="139" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B139" s="100"/>
     </row>
-    <row r="140" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B140" s="100"/>
     </row>
-    <row r="141" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B141" s="100"/>
     </row>
-    <row r="142" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B142" s="100"/>
     </row>
-    <row r="143" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="144" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="145" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="146" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="147" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="148" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="149" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="150" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="151" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="152" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="153" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="154" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="155" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="156" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B156" s="35" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="157" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="158" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="159" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="160" spans="2:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="161" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="162" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="163" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="164" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="165" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="166" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="167" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="168" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="169" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="170" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B170" s="100" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="171" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="172" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="173" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="174" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="175" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="176" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A176" s="35" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="177" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="178" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A178" s="33" t="s">
         <v>270</v>
       </c>
@@ -9153,123 +9153,123 @@
         <v>271</v>
       </c>
     </row>
-    <row r="179" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="180" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="181" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="182" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A182" s="35" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="183" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="193" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="194" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="195" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="196" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="197" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="198" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="199" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="200" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="201" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="202" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="203" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="204" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="205" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="206" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="207" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="208" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="209" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="210" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="211" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="212" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="213" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="214" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="215" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="216" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="217" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="218" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="219" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="220" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="221" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="222" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="223" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="224" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="225" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="226" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="227" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="228" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="229" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="230" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="231" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="232" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="233" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="234" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="235" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="236" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="237" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="238" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="239" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="240" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="241" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="242" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="243" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="244" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="245" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="246" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="247" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="248" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="249" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="250" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="251" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="252" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="253" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="254" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="255" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="256" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="257" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="258" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="259" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="260" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="261" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="262" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="263" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="264" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="265" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="266" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="267" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="268" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="269" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="270" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="271" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="272" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="273" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="274" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="275" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="276" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="277" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="278" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="279" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="280" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="281" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="282" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="283" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="284" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="285" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="286" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="287" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="288" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="289" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="290" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="291" s="35" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="184" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="185" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="186" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="187" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="188" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="189" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="190" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="191" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="192" spans="1:2" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="193" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="194" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="195" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="196" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="197" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="198" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="199" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="200" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="201" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="202" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="203" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="204" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="205" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="206" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="207" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="208" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="209" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="210" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="211" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="212" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="213" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="214" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="215" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="216" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="217" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="218" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="219" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="220" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="221" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="222" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="223" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="224" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="225" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="226" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="227" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="228" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="229" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="230" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="231" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="232" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="233" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="234" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="235" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="236" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="237" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="238" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="239" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="240" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="241" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="242" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="243" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="244" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="245" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="246" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="247" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="248" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="249" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="250" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="251" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="252" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="253" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="254" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="255" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="256" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="257" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="258" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="259" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="260" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="261" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="262" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="263" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="264" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="265" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="266" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="267" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="268" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="269" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="270" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="271" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="272" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="273" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="274" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="275" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="276" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="277" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="278" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="279" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="280" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="281" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="282" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="283" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="284" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="285" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="286" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="287" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="288" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="289" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="290" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="291" s="35" customFormat="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="E15:G15"/>

</xml_diff>